<commit_message>
Rullgardin for Roll i excelmallen
Roll-kolumnen (F2:F200) har nu en riktig datavalidering i Excel med de
fyra rollerna, i stallet for bara en beskrivning i instruktionsbladet.
Ett okant varde gor att raden hoppas over vid import, sa det ar vart att
forhindra felstavningar vid kallan.

- Lista: Funktionar, Domare, Sektionsledare, Tavlingsledare
- Tomt tillatet — da anvands rollen som valts i appen fore importen
- Hjalptext visas nar cellen markeras
- Varning (inte hard blockering) vid varde utanfor listan, sa den som
  klistrar in data fran annat hall inte koras fast
- Instruktionsbladet listar nu rollerna explicit, i samma format som
  kompetenslistan

Verifierat att alla fyra rullgardinsvarden tolkas korrekt av tolkaRoll.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/funktionarer-mall.xlsx
+++ b/public/funktionarer-mall.xlsx
@@ -603,6 +603,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltig roll" error="Välj en av: Funktionär, Domare, Sektionsledare, Tävlingsledare — eller lämna tomt." promptTitle="Roll" prompt="Välj roll. Lämnas fältet tomt används den roll du väljer i appen före importen." type="list" errorStyle="warning">
+      <formula1>"Funktionär,Domare,Sektionsledare,Tävlingsledare"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -613,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -735,35 +740,34 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Funktionär, Domare, Sektionsledare eller Tävlingsledare. Lämnas tom används rollen som valts i appen före importen.</t>
+          <t>En av värdena nedan. Lämnas tom används rollen som valts i appen.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Funktionär, Domare, Sektionsledare, Tävlingsledare</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>TIPS</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>• Rad 2–3 i fliken Funktionärer är exempelrader – ta bort dem eller skriv över dem.</t>
-        </is>
-      </c>
+      <c r="B15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>• Kolumnrubriker måste stå på rad 1, i valfri ordning.</t>
+          <t>• Rad 2–3 i fliken Funktionärer är exempelrader – ta bort dem eller skriv över dem.</t>
         </is>
       </c>
     </row>
@@ -771,7 +775,7 @@
       <c r="A17" s="4" t="inlineStr"/>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>• Filen får vara max 5 MB och ha ändelsen .xlsx eller .xls.</t>
+          <t>• Kolumnrubriker måste stå på rad 1, i valfri ordning.</t>
         </is>
       </c>
     </row>
@@ -779,7 +783,7 @@
       <c r="A18" s="4" t="inlineStr"/>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>• Funktionärer som redan finns i systemet hoppas över.</t>
+          <t>• Filen får vara max 5 MB och ha ändelsen .xlsx eller .xls.</t>
         </is>
       </c>
     </row>
@@ -787,12 +791,20 @@
       <c r="A19" s="4" t="inlineStr"/>
       <c r="B19" s="5" t="inlineStr">
         <is>
+          <t>• Funktionärer som redan finns i systemet hoppas över.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
           <t>• Varje ny funktionär får ett inbjudningsmail automatiskt.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="10" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>• Ett okänt värde i Roll gör att raden hoppas över — den gissas inte.</t>
         </is>

</xml_diff>